<commit_message>
report: refresh sample to template-based version (orange + legend)
</commit_message>
<xml_diff>
--- a/balance_outgoing_mailer/SAMPLE_BALANCE_OUTGOING_20260624.xlsx
+++ b/balance_outgoing_mailer/SAMPLE_BALANCE_OUTGOING_20260624.xlsx
@@ -11,15 +11,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PH0624" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OS0624" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'IP0624'!$A$1:$AA$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'PH0624'!$A$1:$AA$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'OS0624'!$A$1:$AA$12</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$-421]dddd\,\ dd\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="#,###"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,23 +35,46 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color theme="1"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <sz val="9"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -53,36 +83,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A5F"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4B6AE"/>
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE9CF"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE3B4"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8EEF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CDEBD6"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -91,22 +121,37 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00B7BFC9"/>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color rgb="00B7BFC9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B7BFC9"/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color rgb="00B7BFC9"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00B7BFC9"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
@@ -114,11 +159,106 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00B7BFC9"/>
+      <left style="medium">
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color rgb="00B7BFC9"/>
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
       </right>
       <top/>
       <bottom/>
@@ -126,57 +266,425 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B7BFC9"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color rgb="00B7BFC9"/>
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="00B7BFC9"/>
+        <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dashed">
+        <color indexed="64"/>
+      </top>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="dotted">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="dotted">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color indexed="64"/>
+      </left>
+      <right style="dotted">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -253,6 +761,96 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -542,422 +1140,500 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6.7" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7.5" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="6.6640625" customWidth="1" min="1" max="1"/>
+    <col width="6.33203125" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="38.33203125" customWidth="1" min="4" max="4"/>
+    <col width="12.6640625" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17.5" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="3" customWidth="1" min="21" max="21"/>
-    <col width="3" customWidth="1" min="22" max="22"/>
-    <col width="3" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="19.33203125" customWidth="1" min="8" max="8"/>
+    <col width="4.83203125" customWidth="1" min="9" max="9"/>
+    <col width="8.33203125" customWidth="1" min="10" max="10"/>
+    <col width="6.6640625" customWidth="1" min="11" max="11"/>
+    <col width="6.6640625" customWidth="1" min="21" max="21"/>
+    <col width="10.6640625" customWidth="1" min="24" max="24"/>
+    <col width="33.6640625" customWidth="1" min="25" max="25"/>
+    <col width="9.6640625" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>BALANCE OUTGOING MARKET</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="n"/>
+      <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="n"/>
+      <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="3" t="n"/>
+      <c r="R1" s="3" t="n"/>
+      <c r="S1" s="3" t="n"/>
+      <c r="T1" s="3" t="n"/>
+      <c r="U1" s="3" t="n"/>
+      <c r="V1" s="3" t="n"/>
+      <c r="W1" s="3" t="n"/>
+      <c r="X1" s="4" t="n">
+        <v>46197</v>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="12" customHeight="1">
+      <c r="A2" s="5" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="6" t="n"/>
+      <c r="V2" s="6" t="n"/>
+      <c r="W2" s="6" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="12" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>PLANT</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>ITEM CLASS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>LINE</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>MODEL</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>STYLE</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>COLOR</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>IP SPRAY (BEM)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>PAD PRINTING (BEP)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>GEN</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>JUN'26</t>
-        </is>
-      </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>JUNE'26</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
+      <c r="O3" s="11" t="n"/>
+      <c r="P3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
+      <c r="T3" s="10" t="n"/>
+      <c r="U3" s="10" t="n"/>
+      <c r="V3" s="12" t="n"/>
+      <c r="W3" s="13" t="n"/>
+      <c r="X3" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="Y3" s="14" t="inlineStr">
         <is>
           <t>ISSUE</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Z3" s="15" t="inlineStr">
         <is>
           <t>SCAN BEM/BEP</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="16" t="inlineStr">
         <is>
           <t>SCAN DI CKP</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="J4" s="4" t="n">
+    <row r="4" ht="12" customHeight="1">
+      <c r="A4" s="17" t="n"/>
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="19" t="n">
         <v>2</v>
       </c>
+      <c r="U4" s="19" t="n"/>
+      <c r="V4" s="19" t="n"/>
+      <c r="W4" s="19" t="n"/>
+      <c r="X4" s="18" t="n"/>
+      <c r="Y4" s="20" t="n"/>
+      <c r="Z4" s="21" t="n"/>
+      <c r="AA4" s="22" t="n"/>
     </row>
-    <row r="5">
-      <c r="J5" s="4" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1">
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>D+3</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>D+2</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>D+1</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>DD</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="25" t="inlineStr">
         <is>
           <t>D-1</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="25" t="inlineStr">
         <is>
           <t>D-2</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="P5" s="26" t="inlineStr">
         <is>
           <t>D-3</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q5" s="26" t="inlineStr">
         <is>
           <t>D-4</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R5" s="27" t="inlineStr">
         <is>
           <t>D-5</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S5" s="27" t="inlineStr">
         <is>
           <t>D-6</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T5" s="27" t="inlineStr">
         <is>
           <t>D-7</t>
         </is>
       </c>
+      <c r="U5" s="27" t="n"/>
+      <c r="V5" s="27" t="n"/>
+      <c r="W5" s="27" t="n"/>
+      <c r="X5" s="24" t="n"/>
+      <c r="Y5" s="28" t="n"/>
+      <c r="Z5" s="29" t="n"/>
+      <c r="AA5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>3120</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>IP01</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>FGA04</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>AIR MAX 2017 (M)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>849559-405</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="32" t="n"/>
+      <c r="H6" s="32" t="n"/>
+      <c r="I6" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="7" t="n">
+      <c r="J6" s="34" t="n"/>
+      <c r="K6" s="34" t="n">
         <v>180</v>
       </c>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="5" t="n"/>
-      <c r="X6" s="8" t="n">
+      <c r="L6" s="34" t="n"/>
+      <c r="M6" s="34" t="n"/>
+      <c r="N6" s="34" t="n"/>
+      <c r="O6" s="34" t="n"/>
+      <c r="P6" s="34" t="n"/>
+      <c r="Q6" s="34" t="n"/>
+      <c r="R6" s="34" t="n"/>
+      <c r="S6" s="34" t="n"/>
+      <c r="T6" s="34" t="n"/>
+      <c r="U6" s="34" t="n"/>
+      <c r="V6" s="35" t="n"/>
+      <c r="W6" s="35" t="n"/>
+      <c r="X6" s="36" t="n">
         <v>180</v>
       </c>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
+      <c r="Y6" s="37" t="n"/>
+      <c r="Z6" s="32" t="n"/>
+      <c r="AA6" s="38" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="39" t="n"/>
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>II01</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>FGA05</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="33" t="inlineStr">
         <is>
           <t>AIR MAX 90 LTR (TD)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="33" t="inlineStr">
         <is>
           <t>CD6868-100</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="inlineStr">
         <is>
           <t>TD</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="7" t="n">
+      <c r="J7" s="34" t="n"/>
+      <c r="K7" s="34" t="n"/>
+      <c r="L7" s="34" t="n">
         <v>128</v>
       </c>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="8" t="n">
+      <c r="M7" s="34" t="n"/>
+      <c r="N7" s="34" t="n"/>
+      <c r="O7" s="34" t="n"/>
+      <c r="P7" s="34" t="n"/>
+      <c r="Q7" s="34" t="n"/>
+      <c r="R7" s="34" t="n"/>
+      <c r="S7" s="34" t="n"/>
+      <c r="T7" s="34" t="n"/>
+      <c r="U7" s="34" t="n"/>
+      <c r="V7" s="35" t="n"/>
+      <c r="W7" s="35" t="n"/>
+      <c r="X7" s="36" t="n">
         <v>128</v>
       </c>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
+      <c r="Y7" s="37" t="n"/>
+      <c r="Z7" s="32" t="n"/>
+      <c r="AA7" s="38" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="40" t="n"/>
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>II01</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>FGA20</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="42" t="inlineStr">
         <is>
           <t>FREE METCON 7 (W)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="42" t="inlineStr">
         <is>
           <t>II7406-002</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="F8" s="41" t="n"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="41" t="inlineStr">
         <is>
           <t>WO</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="11" t="n">
+      <c r="J8" s="43" t="n"/>
+      <c r="K8" s="43" t="n"/>
+      <c r="L8" s="43" t="n"/>
+      <c r="M8" s="43" t="n">
         <v>2553</v>
       </c>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
-      <c r="T8" s="5" t="n"/>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="8" t="n">
+      <c r="N8" s="43" t="n"/>
+      <c r="O8" s="43" t="n"/>
+      <c r="P8" s="43" t="n"/>
+      <c r="Q8" s="43" t="n"/>
+      <c r="R8" s="43" t="n"/>
+      <c r="S8" s="43" t="n"/>
+      <c r="T8" s="43" t="n"/>
+      <c r="U8" s="43" t="n"/>
+      <c r="V8" s="44" t="n"/>
+      <c r="W8" s="44" t="n"/>
+      <c r="X8" s="41" t="n">
         <v>2553</v>
       </c>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n">
+      <c r="Y8" s="45" t="n"/>
+      <c r="Z8" s="45" t="n">
         <v>1200</v>
       </c>
-      <c r="AA8" s="5" t="n"/>
+      <c r="AA8" s="46" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="12" t="n"/>
-      <c r="K9" s="12" t="n">
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="48" t="n"/>
+      <c r="J9" s="49" t="n"/>
+      <c r="K9" s="49" t="n">
         <v>180</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="49" t="n">
         <v>128</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="M9" s="49" t="n">
         <v>2553</v>
       </c>
-      <c r="N9" s="12" t="n"/>
-      <c r="O9" s="12" t="n"/>
-      <c r="P9" s="12" t="n"/>
-      <c r="Q9" s="12" t="n"/>
-      <c r="R9" s="12" t="n"/>
-      <c r="S9" s="12" t="n"/>
-      <c r="T9" s="12" t="n"/>
-      <c r="U9" s="13" t="n"/>
-      <c r="V9" s="13" t="n"/>
-      <c r="W9" s="13" t="n"/>
-      <c r="X9" s="8" t="n">
+      <c r="N9" s="49" t="n"/>
+      <c r="O9" s="49" t="n"/>
+      <c r="P9" s="49" t="n"/>
+      <c r="Q9" s="49" t="n"/>
+      <c r="R9" s="49" t="n"/>
+      <c r="S9" s="49" t="n"/>
+      <c r="T9" s="49" t="n"/>
+      <c r="U9" s="49" t="n"/>
+      <c r="V9" s="49" t="n"/>
+      <c r="W9" s="49" t="n"/>
+      <c r="X9" s="49" t="n">
         <v>2861</v>
       </c>
-      <c r="Y9" s="13" t="n"/>
-      <c r="Z9" s="13" t="n"/>
-      <c r="AA9" s="13" t="n"/>
+      <c r="Y9" s="50" t="n"/>
+      <c r="Z9" s="50" t="n"/>
+      <c r="AA9" s="50" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -965,22 +1641,24 @@
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="H3:H5"/>
     <mergeCell ref="A6:A8"/>
-    <mergeCell ref="J3:T3"/>
     <mergeCell ref="X3:X5"/>
     <mergeCell ref="C3:C5"/>
+    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="A3:A5"/>
+    <mergeCell ref="E3:E5"/>
     <mergeCell ref="G3:G5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="A9:I9"/>
     <mergeCell ref="F3:F5"/>
-    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="J3:S3"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="D3:D5"/>
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="Z3:Z5"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -988,273 +1666,353 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6.7" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7.5" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="6.6640625" customWidth="1" min="1" max="1"/>
+    <col width="6.33203125" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="38.33203125" customWidth="1" min="4" max="4"/>
+    <col width="12.6640625" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17.5" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="3" customWidth="1" min="21" max="21"/>
-    <col width="3" customWidth="1" min="22" max="22"/>
-    <col width="3" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="19.33203125" customWidth="1" min="8" max="8"/>
+    <col width="4.83203125" customWidth="1" min="9" max="9"/>
+    <col width="8.33203125" customWidth="1" min="10" max="10"/>
+    <col width="6.6640625" customWidth="1" min="11" max="11"/>
+    <col width="6.6640625" customWidth="1" min="21" max="21"/>
+    <col width="10.6640625" customWidth="1" min="24" max="24"/>
+    <col width="33.6640625" customWidth="1" min="25" max="25"/>
+    <col width="9.6640625" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>BALANCE OUTGOING MARKET</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="n"/>
+      <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="n"/>
+      <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="3" t="n"/>
+      <c r="R1" s="3" t="n"/>
+      <c r="S1" s="3" t="n"/>
+      <c r="T1" s="3" t="n"/>
+      <c r="U1" s="3" t="n"/>
+      <c r="V1" s="3" t="n"/>
+      <c r="W1" s="3" t="n"/>
+      <c r="X1" s="4" t="n">
+        <v>46197</v>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="12" customHeight="1">
+      <c r="A2" s="5" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="6" t="n"/>
+      <c r="V2" s="6" t="n"/>
+      <c r="W2" s="6" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="12" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>PLANT</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>ITEM CLASS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>LINE</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>MODEL</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>STYLE</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>COLOR</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>IP SPRAY (BEM)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>PAD PRINTING (BEP)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>GEN</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>JUN'26</t>
-        </is>
-      </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>JUNE'26</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
+      <c r="O3" s="11" t="n"/>
+      <c r="P3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
+      <c r="T3" s="10" t="n"/>
+      <c r="U3" s="10" t="n"/>
+      <c r="V3" s="12" t="n"/>
+      <c r="W3" s="13" t="n"/>
+      <c r="X3" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="Y3" s="14" t="inlineStr">
         <is>
           <t>ISSUE</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Z3" s="15" t="inlineStr">
         <is>
           <t>SCAN BEM/BEP</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="16" t="inlineStr">
         <is>
           <t>SCAN DI CKP</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="J4" s="4" t="n">
+    <row r="4" ht="12" customHeight="1">
+      <c r="A4" s="17" t="n"/>
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="19" t="n">
         <v>2</v>
       </c>
+      <c r="U4" s="19" t="n"/>
+      <c r="V4" s="19" t="n"/>
+      <c r="W4" s="19" t="n"/>
+      <c r="X4" s="18" t="n"/>
+      <c r="Y4" s="20" t="n"/>
+      <c r="Z4" s="21" t="n"/>
+      <c r="AA4" s="22" t="n"/>
     </row>
-    <row r="5">
-      <c r="J5" s="4" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1">
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>D+3</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>D+2</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>D+1</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>DD</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="25" t="inlineStr">
         <is>
           <t>D-1</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="25" t="inlineStr">
         <is>
           <t>D-2</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="P5" s="26" t="inlineStr">
         <is>
           <t>D-3</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q5" s="26" t="inlineStr">
         <is>
           <t>D-4</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R5" s="27" t="inlineStr">
         <is>
           <t>D-5</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S5" s="27" t="inlineStr">
         <is>
           <t>D-6</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T5" s="27" t="inlineStr">
         <is>
           <t>D-7</t>
         </is>
       </c>
+      <c r="U5" s="27" t="n"/>
+      <c r="V5" s="27" t="n"/>
+      <c r="W5" s="27" t="n"/>
+      <c r="X5" s="24" t="n"/>
+      <c r="Y5" s="28" t="n"/>
+      <c r="Z5" s="29" t="n"/>
+      <c r="AA5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n"/>
-      <c r="C6" s="13" t="n"/>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n"/>
-      <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
-      <c r="I6" s="13" t="n"/>
-      <c r="J6" s="12" t="n"/>
-      <c r="K6" s="12" t="n"/>
-      <c r="L6" s="12" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="12" t="n"/>
-      <c r="O6" s="12" t="n"/>
-      <c r="P6" s="12" t="n"/>
-      <c r="Q6" s="12" t="n"/>
-      <c r="R6" s="12" t="n"/>
-      <c r="S6" s="12" t="n"/>
-      <c r="T6" s="12" t="n"/>
-      <c r="U6" s="13" t="n"/>
-      <c r="V6" s="13" t="n"/>
-      <c r="W6" s="13" t="n"/>
-      <c r="X6" s="8" t="n">
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="48" t="n"/>
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+      <c r="M6" s="49" t="n"/>
+      <c r="N6" s="49" t="n"/>
+      <c r="O6" s="49" t="n"/>
+      <c r="P6" s="49" t="n"/>
+      <c r="Q6" s="49" t="n"/>
+      <c r="R6" s="49" t="n"/>
+      <c r="S6" s="49" t="n"/>
+      <c r="T6" s="49" t="n"/>
+      <c r="U6" s="49" t="n"/>
+      <c r="V6" s="49" t="n"/>
+      <c r="W6" s="49" t="n"/>
+      <c r="X6" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="Y6" s="13" t="n"/>
-      <c r="Z6" s="13" t="n"/>
-      <c r="AA6" s="13" t="n"/>
+      <c r="Y6" s="50" t="n"/>
+      <c r="Z6" s="50" t="n"/>
+      <c r="AA6" s="50" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="X1:AA2"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="H3:H5"/>
-    <mergeCell ref="J3:T3"/>
     <mergeCell ref="X3:X5"/>
     <mergeCell ref="C3:C5"/>
+    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="A3:A5"/>
+    <mergeCell ref="E3:E5"/>
     <mergeCell ref="G3:G5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="F3:F5"/>
-    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="J3:S3"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="D3:D5"/>
     <mergeCell ref="A6:I6"/>
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="Z3:Z5"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1262,619 +2020,699 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6.7" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7.5" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="6.6640625" customWidth="1" min="1" max="1"/>
+    <col width="6.33203125" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="38.33203125" customWidth="1" min="4" max="4"/>
+    <col width="12.6640625" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="17.5" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="3" customWidth="1" min="21" max="21"/>
-    <col width="3" customWidth="1" min="22" max="22"/>
-    <col width="3" customWidth="1" min="23" max="23"/>
-    <col width="10" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="19.33203125" customWidth="1" min="8" max="8"/>
+    <col width="4.83203125" customWidth="1" min="9" max="9"/>
+    <col width="8.33203125" customWidth="1" min="10" max="10"/>
+    <col width="6.6640625" customWidth="1" min="11" max="11"/>
+    <col width="6.6640625" customWidth="1" min="21" max="21"/>
+    <col width="10.6640625" customWidth="1" min="24" max="24"/>
+    <col width="33.6640625" customWidth="1" min="25" max="25"/>
+    <col width="9.6640625" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="12" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>BALANCE OUTGOING MARKET</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+      <c r="H1" s="3" t="n"/>
+      <c r="I1" s="3" t="n"/>
+      <c r="J1" s="3" t="n"/>
+      <c r="K1" s="3" t="n"/>
+      <c r="L1" s="3" t="n"/>
+      <c r="M1" s="3" t="n"/>
+      <c r="N1" s="3" t="n"/>
+      <c r="O1" s="3" t="n"/>
+      <c r="P1" s="3" t="n"/>
+      <c r="Q1" s="3" t="n"/>
+      <c r="R1" s="3" t="n"/>
+      <c r="S1" s="3" t="n"/>
+      <c r="T1" s="3" t="n"/>
+      <c r="U1" s="3" t="n"/>
+      <c r="V1" s="3" t="n"/>
+      <c r="W1" s="3" t="n"/>
+      <c r="X1" s="4" t="n">
+        <v>46197</v>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="2" ht="12" customHeight="1">
+      <c r="A2" s="5" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="6" t="n"/>
+      <c r="R2" s="6" t="n"/>
+      <c r="S2" s="6" t="n"/>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="6" t="n"/>
+      <c r="V2" s="6" t="n"/>
+      <c r="W2" s="6" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="12" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>PLANT</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>ITEM CLASS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>LINE</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>MODEL</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>STYLE</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>COLOR</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>IP SPRAY (BEM)</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>PAD PRINTING (BEP)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>GEN</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>JUN'26</t>
-        </is>
-      </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>JUNE'26</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
+      <c r="N3" s="11" t="n"/>
+      <c r="O3" s="11" t="n"/>
+      <c r="P3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
+      <c r="S3" s="11" t="n"/>
+      <c r="T3" s="10" t="n"/>
+      <c r="U3" s="10" t="n"/>
+      <c r="V3" s="12" t="n"/>
+      <c r="W3" s="13" t="n"/>
+      <c r="X3" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
+      <c r="Y3" s="14" t="inlineStr">
         <is>
           <t>ISSUE</t>
         </is>
       </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Z3" s="15" t="inlineStr">
         <is>
           <t>SCAN BEM/BEP</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="16" t="inlineStr">
         <is>
           <t>SCAN DI CKP</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="J4" s="4" t="n">
+    <row r="4" ht="12" customHeight="1">
+      <c r="A4" s="17" t="n"/>
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="18" t="n"/>
+      <c r="J4" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="19" t="n">
         <v>22</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="19" t="n">
         <v>24</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="19" t="n">
         <v>2</v>
       </c>
+      <c r="U4" s="19" t="n"/>
+      <c r="V4" s="19" t="n"/>
+      <c r="W4" s="19" t="n"/>
+      <c r="X4" s="18" t="n"/>
+      <c r="Y4" s="20" t="n"/>
+      <c r="Z4" s="21" t="n"/>
+      <c r="AA4" s="22" t="n"/>
     </row>
-    <row r="5">
-      <c r="J5" s="4" t="inlineStr">
+    <row r="5" ht="16.5" customHeight="1">
+      <c r="A5" s="23" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="25" t="inlineStr">
         <is>
           <t>D+3</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="25" t="inlineStr">
         <is>
           <t>D+2</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="25" t="inlineStr">
         <is>
           <t>D+1</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="25" t="inlineStr">
         <is>
           <t>DD</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="N5" s="25" t="inlineStr">
         <is>
           <t>D-1</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O5" s="25" t="inlineStr">
         <is>
           <t>D-2</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="P5" s="26" t="inlineStr">
         <is>
           <t>D-3</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q5" s="26" t="inlineStr">
         <is>
           <t>D-4</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R5" s="27" t="inlineStr">
         <is>
           <t>D-5</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S5" s="27" t="inlineStr">
         <is>
           <t>D-6</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T5" s="27" t="inlineStr">
         <is>
           <t>D-7</t>
         </is>
       </c>
+      <c r="U5" s="27" t="n"/>
+      <c r="V5" s="27" t="n"/>
+      <c r="W5" s="27" t="n"/>
+      <c r="X5" s="24" t="n"/>
+      <c r="Y5" s="28" t="n"/>
+      <c r="Z5" s="29" t="n"/>
+      <c r="AA5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>OS01</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>FGA01</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="33" t="inlineStr">
         <is>
           <t>AIR MAX 90 RECRAFT (M)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>CN8490-003</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="32" t="n"/>
+      <c r="H6" s="32" t="n"/>
+      <c r="I6" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
-      <c r="M6" s="11" t="n">
+      <c r="J6" s="34" t="n"/>
+      <c r="K6" s="34" t="n"/>
+      <c r="L6" s="34" t="n"/>
+      <c r="M6" s="34" t="n">
         <v>2297</v>
       </c>
-      <c r="N6" s="14" t="n">
+      <c r="N6" s="34" t="n">
         <v>2189</v>
       </c>
-      <c r="O6" s="14" t="n">
+      <c r="O6" s="34" t="n">
         <v>1404</v>
       </c>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
-      <c r="S6" s="5" t="n"/>
-      <c r="T6" s="5" t="n"/>
-      <c r="U6" s="5" t="n"/>
-      <c r="V6" s="5" t="n"/>
-      <c r="W6" s="5" t="n"/>
-      <c r="X6" s="8" t="n">
+      <c r="P6" s="34" t="n"/>
+      <c r="Q6" s="34" t="n"/>
+      <c r="R6" s="34" t="n"/>
+      <c r="S6" s="34" t="n"/>
+      <c r="T6" s="34" t="n"/>
+      <c r="U6" s="34" t="n"/>
+      <c r="V6" s="35" t="n"/>
+      <c r="W6" s="35" t="n"/>
+      <c r="X6" s="36" t="n">
         <v>5890</v>
       </c>
-      <c r="Y6" s="5" t="n"/>
-      <c r="Z6" s="5" t="n"/>
-      <c r="AA6" s="5" t="n"/>
+      <c r="Y6" s="37" t="n"/>
+      <c r="Z6" s="32" t="n"/>
+      <c r="AA6" s="38" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="39" t="n"/>
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>OS01</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>FGA01</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="33" t="inlineStr">
         <is>
           <t>AIR MAX 90 RECRAFT (M)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="33" t="inlineStr">
         <is>
           <t>CN8490-100</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="7" t="n">
+      <c r="J7" s="34" t="n"/>
+      <c r="K7" s="34" t="n">
         <v>2224</v>
       </c>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
-      <c r="S7" s="5" t="n"/>
-      <c r="T7" s="5" t="n"/>
-      <c r="U7" s="5" t="n"/>
-      <c r="V7" s="5" t="n"/>
-      <c r="W7" s="5" t="n"/>
-      <c r="X7" s="8" t="n">
+      <c r="L7" s="34" t="n"/>
+      <c r="M7" s="34" t="n"/>
+      <c r="N7" s="34" t="n"/>
+      <c r="O7" s="34" t="n"/>
+      <c r="P7" s="34" t="n"/>
+      <c r="Q7" s="34" t="n"/>
+      <c r="R7" s="34" t="n"/>
+      <c r="S7" s="34" t="n"/>
+      <c r="T7" s="34" t="n"/>
+      <c r="U7" s="34" t="n"/>
+      <c r="V7" s="35" t="n"/>
+      <c r="W7" s="35" t="n"/>
+      <c r="X7" s="36" t="n">
         <v>2224</v>
       </c>
-      <c r="Y7" s="5" t="n"/>
-      <c r="Z7" s="5" t="n"/>
-      <c r="AA7" s="5" t="n"/>
+      <c r="Y7" s="37" t="n"/>
+      <c r="Z7" s="32" t="n"/>
+      <c r="AA7" s="38" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="39" t="n"/>
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>OS01</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>FGA02</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>AIR MAX 90 RECRAFT (M)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="33" t="inlineStr">
         <is>
           <t>CN8490-003</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="F8" s="32" t="n"/>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="7" t="n">
+      <c r="J8" s="34" t="n"/>
+      <c r="K8" s="34" t="n">
         <v>2280</v>
       </c>
-      <c r="L8" s="5" t="n"/>
-      <c r="M8" s="5" t="n"/>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
-      <c r="S8" s="5" t="n"/>
-      <c r="T8" s="5" t="n"/>
-      <c r="U8" s="5" t="n"/>
-      <c r="V8" s="5" t="n"/>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="8" t="n">
+      <c r="L8" s="34" t="n"/>
+      <c r="M8" s="34" t="n"/>
+      <c r="N8" s="34" t="n"/>
+      <c r="O8" s="34" t="n"/>
+      <c r="P8" s="34" t="n"/>
+      <c r="Q8" s="34" t="n"/>
+      <c r="R8" s="34" t="n"/>
+      <c r="S8" s="34" t="n"/>
+      <c r="T8" s="34" t="n"/>
+      <c r="U8" s="34" t="n"/>
+      <c r="V8" s="35" t="n"/>
+      <c r="W8" s="35" t="n"/>
+      <c r="X8" s="36" t="n">
         <v>2280</v>
       </c>
-      <c r="Y8" s="5" t="n"/>
-      <c r="Z8" s="5" t="n"/>
-      <c r="AA8" s="5" t="n"/>
+      <c r="Y8" s="37" t="n"/>
+      <c r="Z8" s="32" t="n"/>
+      <c r="AA8" s="38" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="40" t="n"/>
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>OS01</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>FGA03</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="33" t="inlineStr">
         <is>
           <t>P-6000 (M)</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="33" t="inlineStr">
         <is>
           <t>CD6404-107</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="F9" s="32" t="n"/>
+      <c r="G9" s="32" t="n"/>
+      <c r="H9" s="32" t="n"/>
+      <c r="I9" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="7" t="n">
+      <c r="J9" s="34" t="n"/>
+      <c r="K9" s="34" t="n"/>
+      <c r="L9" s="34" t="n">
         <v>3325</v>
       </c>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
-      <c r="S9" s="5" t="n"/>
-      <c r="T9" s="5" t="n"/>
-      <c r="U9" s="5" t="n"/>
-      <c r="V9" s="5" t="n"/>
-      <c r="W9" s="5" t="n"/>
-      <c r="X9" s="8" t="n">
+      <c r="M9" s="34" t="n"/>
+      <c r="N9" s="34" t="n"/>
+      <c r="O9" s="34" t="n"/>
+      <c r="P9" s="34" t="n"/>
+      <c r="Q9" s="34" t="n"/>
+      <c r="R9" s="34" t="n"/>
+      <c r="S9" s="34" t="n"/>
+      <c r="T9" s="34" t="n"/>
+      <c r="U9" s="34" t="n"/>
+      <c r="V9" s="35" t="n"/>
+      <c r="W9" s="35" t="n"/>
+      <c r="X9" s="36" t="n">
         <v>3325</v>
       </c>
-      <c r="Y9" s="5" t="n"/>
-      <c r="Z9" s="5" t="n">
+      <c r="Y9" s="37" t="n"/>
+      <c r="Z9" s="32" t="n">
         <v>4100</v>
       </c>
-      <c r="AA9" s="5" t="n"/>
+      <c r="AA9" s="38" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="32" t="inlineStr">
         <is>
           <t>OS01</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>FGA22</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="33" t="inlineStr">
         <is>
           <t>ZOOM VOMERO 5 (M)</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="33" t="inlineStr">
         <is>
           <t>IM3486-003</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
       </c>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="14" t="n">
+      <c r="J10" s="34" t="n"/>
+      <c r="K10" s="34" t="n"/>
+      <c r="L10" s="34" t="n"/>
+      <c r="M10" s="34" t="n"/>
+      <c r="N10" s="34" t="n">
         <v>2568</v>
       </c>
-      <c r="O10" s="5" t="n"/>
-      <c r="P10" s="5" t="n"/>
-      <c r="Q10" s="5" t="n"/>
-      <c r="R10" s="5" t="n"/>
-      <c r="S10" s="5" t="n"/>
-      <c r="T10" s="5" t="n"/>
-      <c r="U10" s="5" t="n"/>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="5" t="n"/>
-      <c r="X10" s="8" t="n">
+      <c r="O10" s="34" t="n"/>
+      <c r="P10" s="34" t="n"/>
+      <c r="Q10" s="34" t="n"/>
+      <c r="R10" s="34" t="n"/>
+      <c r="S10" s="34" t="n"/>
+      <c r="T10" s="34" t="n"/>
+      <c r="U10" s="34" t="n"/>
+      <c r="V10" s="35" t="n"/>
+      <c r="W10" s="35" t="n"/>
+      <c r="X10" s="36" t="n">
         <v>2568</v>
       </c>
-      <c r="Y10" s="5" t="n"/>
-      <c r="Z10" s="5" t="n"/>
-      <c r="AA10" s="5" t="n"/>
+      <c r="Y10" s="37" t="n"/>
+      <c r="Z10" s="32" t="n"/>
+      <c r="AA10" s="38" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>OS03</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>FGA35</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>DOWNSHIFTER 13 (W)</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="42" t="inlineStr">
         <is>
           <t>FD6476-001</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="41" t="n"/>
+      <c r="I11" s="41" t="inlineStr">
         <is>
           <t>WO</t>
         </is>
       </c>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="11" t="n">
+      <c r="J11" s="43" t="n"/>
+      <c r="K11" s="43" t="n"/>
+      <c r="L11" s="43" t="n"/>
+      <c r="M11" s="43" t="n">
         <v>980</v>
       </c>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
-      <c r="P11" s="5" t="n"/>
-      <c r="Q11" s="5" t="n"/>
-      <c r="R11" s="5" t="n"/>
-      <c r="S11" s="5" t="n"/>
-      <c r="T11" s="5" t="n"/>
-      <c r="U11" s="5" t="n"/>
-      <c r="V11" s="5" t="n"/>
-      <c r="W11" s="5" t="n"/>
-      <c r="X11" s="8" t="n">
+      <c r="N11" s="43" t="n"/>
+      <c r="O11" s="43" t="n"/>
+      <c r="P11" s="43" t="n"/>
+      <c r="Q11" s="43" t="n"/>
+      <c r="R11" s="43" t="n"/>
+      <c r="S11" s="43" t="n"/>
+      <c r="T11" s="43" t="n"/>
+      <c r="U11" s="43" t="n"/>
+      <c r="V11" s="44" t="n"/>
+      <c r="W11" s="44" t="n"/>
+      <c r="X11" s="41" t="n">
         <v>980</v>
       </c>
-      <c r="Y11" s="5" t="n"/>
-      <c r="Z11" s="5" t="n"/>
-      <c r="AA11" s="5" t="n"/>
+      <c r="Y11" s="45" t="n"/>
+      <c r="Z11" s="45" t="n"/>
+      <c r="AA11" s="46" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
-      <c r="J12" s="12" t="n"/>
-      <c r="K12" s="12" t="n">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="48" t="n"/>
+      <c r="J12" s="49" t="n"/>
+      <c r="K12" s="49" t="n">
         <v>4504</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="L12" s="49" t="n">
         <v>3325</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="M12" s="49" t="n">
         <v>3277</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="49" t="n">
         <v>4757</v>
       </c>
-      <c r="O12" s="12" t="n">
+      <c r="O12" s="49" t="n">
         <v>1404</v>
       </c>
-      <c r="P12" s="12" t="n"/>
-      <c r="Q12" s="12" t="n"/>
-      <c r="R12" s="12" t="n"/>
-      <c r="S12" s="12" t="n"/>
-      <c r="T12" s="12" t="n"/>
-      <c r="U12" s="13" t="n"/>
-      <c r="V12" s="13" t="n"/>
-      <c r="W12" s="13" t="n"/>
-      <c r="X12" s="8" t="n">
+      <c r="P12" s="49" t="n"/>
+      <c r="Q12" s="49" t="n"/>
+      <c r="R12" s="49" t="n"/>
+      <c r="S12" s="49" t="n"/>
+      <c r="T12" s="49" t="n"/>
+      <c r="U12" s="49" t="n"/>
+      <c r="V12" s="49" t="n"/>
+      <c r="W12" s="49" t="n"/>
+      <c r="X12" s="49" t="n">
         <v>17267</v>
       </c>
-      <c r="Y12" s="13" t="n"/>
-      <c r="Z12" s="13" t="n"/>
-      <c r="AA12" s="13" t="n"/>
+      <c r="Y12" s="50" t="n"/>
+      <c r="Z12" s="50" t="n"/>
+      <c r="AA12" s="50" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="X1:AA2"/>
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="H3:H5"/>
-    <mergeCell ref="J3:T3"/>
     <mergeCell ref="X3:X5"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="A6:A9"/>
+    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="A3:A5"/>
+    <mergeCell ref="E3:E5"/>
     <mergeCell ref="G3:G5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="AA3:AA5"/>
     <mergeCell ref="F3:F5"/>
-    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="J3:S3"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="D3:D5"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="Z3:Z5"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>